<commit_message>
Grafik balonu: hafta tarih aralığıyla (20-26 Eylül 2026)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/agustos/ozdilekteyim-agustos-2026-arama-talebi.xlsx
+++ b/agustos/ozdilekteyim-agustos-2026-arama-talebi.xlsx
@@ -9042,267 +9042,267 @@
       </c>
       <c r="C1" s="8" t="inlineStr">
         <is>
-          <t>31 Ağu 2025 haftası · Trends 0-100 (Google Trends)</t>
+          <t>31 Ağustos - 6 Eylül 2025 · Trends 0-100 (Google Trends)</t>
         </is>
       </c>
       <c r="D1" s="8" t="inlineStr">
         <is>
-          <t>7 Eyl 2025 haftası · Trends 0-100 (Google Trends)</t>
+          <t>7-13 Eylül 2025 · Trends 0-100 (Google Trends)</t>
         </is>
       </c>
       <c r="E1" s="8" t="inlineStr">
         <is>
-          <t>14 Eyl 2025 haftası · Trends 0-100 (Google Trends)</t>
+          <t>14-20 Eylül 2025 · Trends 0-100 (Google Trends)</t>
         </is>
       </c>
       <c r="F1" s="8" t="inlineStr">
         <is>
-          <t>21 Eyl 2025 haftası · Trends 0-100 (Google Trends)</t>
+          <t>21-27 Eylül 2025 · Trends 0-100 (Google Trends)</t>
         </is>
       </c>
       <c r="G1" s="8" t="inlineStr">
         <is>
-          <t>28 Eyl 2025 haftası · Trends 0-100 (Google Trends)</t>
+          <t>28 Eylül - 4 Ekim 2025 · Trends 0-100 (Google Trends)</t>
         </is>
       </c>
       <c r="H1" s="8" t="inlineStr">
         <is>
-          <t>5 Eki 2025 haftası · Trends 0-100 (Google Trends)</t>
+          <t>5-11 Ekim 2025 · Trends 0-100 (Google Trends)</t>
         </is>
       </c>
       <c r="I1" s="8" t="inlineStr">
         <is>
-          <t>12 Eki 2025 haftası · Trends 0-100 (Google Trends)</t>
+          <t>12-18 Ekim 2025 · Trends 0-100 (Google Trends)</t>
         </is>
       </c>
       <c r="J1" s="8" t="inlineStr">
         <is>
-          <t>19 Eki 2025 haftası · Trends 0-100 (Google Trends)</t>
+          <t>19-25 Ekim 2025 · Trends 0-100 (Google Trends)</t>
         </is>
       </c>
       <c r="K1" s="8" t="inlineStr">
         <is>
-          <t>26 Eki 2025 haftası · Trends 0-100 (Google Trends)</t>
+          <t>26 Ekim - 1 Kasım 2025 · Trends 0-100 (Google Trends)</t>
         </is>
       </c>
       <c r="L1" s="8" t="inlineStr">
         <is>
-          <t>2 Kas 2025 haftası · Trends 0-100 (Google Trends)</t>
+          <t>2-8 Kasım 2025 · Trends 0-100 (Google Trends)</t>
         </is>
       </c>
       <c r="M1" s="8" t="inlineStr">
         <is>
-          <t>9 Kas 2025 haftası · Trends 0-100 (Google Trends)</t>
+          <t>9-15 Kasım 2025 · Trends 0-100 (Google Trends)</t>
         </is>
       </c>
       <c r="N1" s="8" t="inlineStr">
         <is>
-          <t>16 Kas 2025 haftası · Trends 0-100 (Google Trends)</t>
+          <t>16-22 Kasım 2025 · Trends 0-100 (Google Trends)</t>
         </is>
       </c>
       <c r="O1" s="8" t="inlineStr">
         <is>
-          <t>23 Kas 2025 haftası · Trends 0-100 (Google Trends)</t>
+          <t>23-29 Kasım 2025 · Trends 0-100 (Google Trends)</t>
         </is>
       </c>
       <c r="P1" s="8" t="inlineStr">
         <is>
-          <t>30 Kas 2025 haftası · Trends 0-100 (Google Trends)</t>
+          <t>30 Kasım - 6 Aralık 2025 · Trends 0-100 (Google Trends)</t>
         </is>
       </c>
       <c r="Q1" s="8" t="inlineStr">
         <is>
-          <t>7 Ara 2025 haftası · Trends 0-100 (Google Trends)</t>
+          <t>7-13 Aralık 2025 · Trends 0-100 (Google Trends)</t>
         </is>
       </c>
       <c r="R1" s="8" t="inlineStr">
         <is>
-          <t>14 Ara 2025 haftası · Trends 0-100 (Google Trends)</t>
+          <t>14-20 Aralık 2025 · Trends 0-100 (Google Trends)</t>
         </is>
       </c>
       <c r="S1" s="8" t="inlineStr">
         <is>
-          <t>21 Ara 2025 haftası · Trends 0-100 (Google Trends)</t>
+          <t>21-27 Aralık 2025 · Trends 0-100 (Google Trends)</t>
         </is>
       </c>
       <c r="T1" s="8" t="inlineStr">
         <is>
-          <t>28 Ara 2025 haftası · Trends 0-100 (Google Trends)</t>
+          <t>28 Aralık 2025 - 3 Ocak 2026 · Trends 0-100 (Google Trends)</t>
         </is>
       </c>
       <c r="U1" s="8" t="inlineStr">
         <is>
-          <t>4 Oca 2026 haftası · Trends 0-100 (Google Trends)</t>
+          <t>4-10 Ocak 2026 · Trends 0-100 (Google Trends)</t>
         </is>
       </c>
       <c r="V1" s="8" t="inlineStr">
         <is>
-          <t>11 Oca 2026 haftası · Trends 0-100 (Google Trends)</t>
+          <t>11-17 Ocak 2026 · Trends 0-100 (Google Trends)</t>
         </is>
       </c>
       <c r="W1" s="8" t="inlineStr">
         <is>
-          <t>18 Oca 2026 haftası · Trends 0-100 (Google Trends)</t>
+          <t>18-24 Ocak 2026 · Trends 0-100 (Google Trends)</t>
         </is>
       </c>
       <c r="X1" s="8" t="inlineStr">
         <is>
-          <t>25 Oca 2026 haftası · Trends 0-100 (Google Trends)</t>
+          <t>25-31 Ocak 2026 · Trends 0-100 (Google Trends)</t>
         </is>
       </c>
       <c r="Y1" s="8" t="inlineStr">
         <is>
-          <t>1 Şub 2026 haftası · Trends 0-100 (Google Trends)</t>
+          <t>1-7 Şubat 2026 · Trends 0-100 (Google Trends)</t>
         </is>
       </c>
       <c r="Z1" s="8" t="inlineStr">
         <is>
-          <t>8 Şub 2026 haftası · Trends 0-100 (Google Trends)</t>
+          <t>8-14 Şubat 2026 · Trends 0-100 (Google Trends)</t>
         </is>
       </c>
       <c r="AA1" s="8" t="inlineStr">
         <is>
-          <t>15 Şub 2026 haftası · Trends 0-100 (Google Trends)</t>
+          <t>15-21 Şubat 2026 · Trends 0-100 (Google Trends)</t>
         </is>
       </c>
       <c r="AB1" s="8" t="inlineStr">
         <is>
-          <t>22 Şub 2026 haftası · Trends 0-100 (Google Trends)</t>
+          <t>22-28 Şubat 2026 · Trends 0-100 (Google Trends)</t>
         </is>
       </c>
       <c r="AC1" s="8" t="inlineStr">
         <is>
-          <t>1 Mar 2026 haftası · Trends 0-100 (Google Trends)</t>
+          <t>1-7 Mart 2026 · Trends 0-100 (Google Trends)</t>
         </is>
       </c>
       <c r="AD1" s="8" t="inlineStr">
         <is>
-          <t>8 Mar 2026 haftası · Trends 0-100 (Google Trends)</t>
+          <t>8-14 Mart 2026 · Trends 0-100 (Google Trends)</t>
         </is>
       </c>
       <c r="AE1" s="8" t="inlineStr">
         <is>
-          <t>15 Mar 2026 haftası · Trends 0-100 (Google Trends)</t>
+          <t>15-21 Mart 2026 · Trends 0-100 (Google Trends)</t>
         </is>
       </c>
       <c r="AF1" s="8" t="inlineStr">
         <is>
-          <t>22 Mar 2026 haftası · Trends 0-100 (Google Trends)</t>
+          <t>22-28 Mart 2026 · Trends 0-100 (Google Trends)</t>
         </is>
       </c>
       <c r="AG1" s="8" t="inlineStr">
         <is>
-          <t>29 Mar 2026 haftası · Trends 0-100 (Google Trends)</t>
+          <t>29 Mart - 4 Nisan 2026 · Trends 0-100 (Google Trends)</t>
         </is>
       </c>
       <c r="AH1" s="8" t="inlineStr">
         <is>
-          <t>5 Nis 2026 haftası · Trends 0-100 (Google Trends)</t>
+          <t>5-11 Nisan 2026 · Trends 0-100 (Google Trends)</t>
         </is>
       </c>
       <c r="AI1" s="8" t="inlineStr">
         <is>
-          <t>12 Nis 2026 haftası · Trends 0-100 (Google Trends)</t>
+          <t>12-18 Nisan 2026 · Trends 0-100 (Google Trends)</t>
         </is>
       </c>
       <c r="AJ1" s="8" t="inlineStr">
         <is>
-          <t>19 Nis 2026 haftası · Trends 0-100 (Google Trends)</t>
+          <t>19-25 Nisan 2026 · Trends 0-100 (Google Trends)</t>
         </is>
       </c>
       <c r="AK1" s="8" t="inlineStr">
         <is>
-          <t>26 Nis 2026 haftası · Trends 0-100 (Google Trends)</t>
+          <t>26 Nisan - 2 Mayıs 2026 · Trends 0-100 (Google Trends)</t>
         </is>
       </c>
       <c r="AL1" s="8" t="inlineStr">
         <is>
-          <t>3 May 2026 haftası · Trends 0-100 (Google Trends)</t>
+          <t>3-9 Mayıs 2026 · Trends 0-100 (Google Trends)</t>
         </is>
       </c>
       <c r="AM1" s="8" t="inlineStr">
         <is>
-          <t>10 May 2026 haftası · Trends 0-100 (Google Trends)</t>
+          <t>10-16 Mayıs 2026 · Trends 0-100 (Google Trends)</t>
         </is>
       </c>
       <c r="AN1" s="8" t="inlineStr">
         <is>
-          <t>17 May 2026 haftası · Trends 0-100 (Google Trends)</t>
+          <t>17-23 Mayıs 2026 · Trends 0-100 (Google Trends)</t>
         </is>
       </c>
       <c r="AO1" s="8" t="inlineStr">
         <is>
-          <t>24 May 2026 haftası · Trends 0-100 (Google Trends)</t>
+          <t>24-30 Mayıs 2026 · Trends 0-100 (Google Trends)</t>
         </is>
       </c>
       <c r="AP1" s="8" t="inlineStr">
         <is>
-          <t>31 May 2026 haftası · Trends 0-100 (Google Trends)</t>
+          <t>31 Mayıs - 6 Haziran 2026 · Trends 0-100 (Google Trends)</t>
         </is>
       </c>
       <c r="AQ1" s="8" t="inlineStr">
         <is>
-          <t>7 Haz 2026 haftası · Trends 0-100 (Google Trends)</t>
+          <t>7-13 Haziran 2026 · Trends 0-100 (Google Trends)</t>
         </is>
       </c>
       <c r="AR1" s="8" t="inlineStr">
         <is>
-          <t>14 Haz 2026 haftası · Trends 0-100 (Google Trends)</t>
+          <t>14-20 Haziran 2026 · Trends 0-100 (Google Trends)</t>
         </is>
       </c>
       <c r="AS1" s="8" t="inlineStr">
         <is>
-          <t>21 Haz 2026 haftası · Trends 0-100 (Google Trends)</t>
+          <t>21-27 Haziran 2026 · Trends 0-100 (Google Trends)</t>
         </is>
       </c>
       <c r="AT1" s="8" t="inlineStr">
         <is>
-          <t>28 Haz 2026 haftası · Trends 0-100 (Google Trends)</t>
+          <t>28 Haziran - 4 Temmuz 2026 · Trends 0-100 (Google Trends)</t>
         </is>
       </c>
       <c r="AU1" s="8" t="inlineStr">
         <is>
-          <t>5 Tem 2026 haftası · Trends 0-100 (Google Trends)</t>
+          <t>5-11 Temmuz 2026 · Trends 0-100 (Google Trends)</t>
         </is>
       </c>
       <c r="AV1" s="8" t="inlineStr">
         <is>
-          <t>12 Tem 2026 haftası · Trends 0-100 (Google Trends)</t>
+          <t>12-18 Temmuz 2026 · Trends 0-100 (Google Trends)</t>
         </is>
       </c>
       <c r="AW1" s="8" t="inlineStr">
         <is>
-          <t>19 Tem 2026 haftası · Trends 0-100 (Google Trends)</t>
+          <t>19-25 Temmuz 2026 · Trends 0-100 (Google Trends)</t>
         </is>
       </c>
       <c r="AX1" s="8" t="inlineStr">
         <is>
-          <t>26 Tem 2026 haftası · Trends 0-100 (Google Trends)</t>
+          <t>26 Temmuz - 1 Ağustos 2026 · Trends 0-100 (Google Trends)</t>
         </is>
       </c>
       <c r="AY1" s="8" t="inlineStr">
         <is>
-          <t>2 Ağu 2026 haftası · Trends 0-100 (Google Trends)</t>
+          <t>2-8 Ağustos 2026 · Trends 0-100 (Google Trends)</t>
         </is>
       </c>
       <c r="AZ1" s="8" t="inlineStr">
         <is>
-          <t>9 Ağu 2026 haftası · Trends 0-100 (Google Trends)</t>
+          <t>9-15 Ağustos 2026 · Trends 0-100 (Google Trends)</t>
         </is>
       </c>
       <c r="BA1" s="8" t="inlineStr">
         <is>
-          <t>16 Ağu 2026 haftası · Trends 0-100 (Google Trends)</t>
+          <t>16-22 Ağustos 2026 · Trends 0-100 (Google Trends)</t>
         </is>
       </c>
       <c r="BB1" s="8" t="inlineStr">
         <is>
-          <t>23 Ağu 2026 haftası · Trends 0-100 (Google Trends)</t>
+          <t>23-29 Ağustos 2026 · Trends 0-100 (Google Trends)</t>
         </is>
       </c>
       <c r="BC1" s="8" t="inlineStr">
         <is>
-          <t>30 Ağu 2026 haftası · Trends 0-100 (Google Trends)</t>
+          <t>30 Ağustos - 5 Eylül 2026 · Trends 0-100 (Google Trends)</t>
         </is>
       </c>
     </row>

</xml_diff>